<commit_message>
Integra Uruguay 2012, documento metodologico y extiende a 36 matrices
- Uruguay 2012 reconstruida desde el COU detallado del BCU (hoja unica COU_C:
  oferta+utilizacion+VA, 134 prod x 107 ind). Parser nuevo
  Codigo/src/parsers/uruguay_cou_2012.py; config uruguay_cou_2012 en main.py y
  mapeo a Uruguay en el generador de paquete. 107 sectores, Leontief OK.
- La serie pasa de 35 a 36 matrices. Regenerado/validado/auditado: 36/36
  estructural OK, 0 sectores de fuente pendientes.
- Argentina 2005-2017 descartado: CEPAL/INDEC solo publican COU 2004, 2018-2021
  (+2022 directo). Documentado en handoff y fuentes.
- Documento metodologico completo en LaTeX/PDF/Word (Metodologia_MIP.{tex,pdf,
  docx}), con notacion del marco CEPAL "MIP Extendida Ambientalmente" e
  inventario de las 36 matrices.
- Docs actualizados: CLAUDE_HANDOFF.md, README.md, FUENTES_EXTERNAS_HISTORICO.md,
  indices, validacion y auditoria.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/indice_matrices.xlsx
+++ b/indice_matrices.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="52">
   <si>
     <t>pais</t>
   </si>
@@ -55,6 +55,9 @@
     <t>mexico</t>
   </si>
   <si>
+    <t>uruguay_cou_2012</t>
+  </si>
+  <si>
     <t>uruguay</t>
   </si>
   <si>
@@ -158,6 +161,9 @@
   </si>
   <si>
     <t>output\matrices_insumo_producto\Mexico\MIP_Mexico_2018.xlsx</t>
+  </si>
+  <si>
+    <t>output\matrices_insumo_producto\Uruguay\MIP_Uruguay_2012.xlsx</t>
   </si>
   <si>
     <t>output\matrices_insumo_producto\Uruguay\MIP_Uruguay_2016.xlsx</t>
@@ -521,7 +527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -549,7 +555,7 @@
         <v>1997</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -563,7 +569,7 @@
         <v>2004</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -577,7 +583,7 @@
         <v>2018</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -591,7 +597,7 @@
         <v>2019</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -605,7 +611,7 @@
         <v>2020</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -619,7 +625,7 @@
         <v>2021</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -633,7 +639,7 @@
         <v>2022</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -647,7 +653,7 @@
         <v>2000</v>
       </c>
       <c r="D9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -661,7 +667,7 @@
         <v>2001</v>
       </c>
       <c r="D10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -675,7 +681,7 @@
         <v>2002</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -689,7 +695,7 @@
         <v>2003</v>
       </c>
       <c r="D12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -703,7 +709,7 @@
         <v>2004</v>
       </c>
       <c r="D13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -717,7 +723,7 @@
         <v>2005</v>
       </c>
       <c r="D14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -731,7 +737,7 @@
         <v>2006</v>
       </c>
       <c r="D15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -745,7 +751,7 @@
         <v>2007</v>
       </c>
       <c r="D16" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -759,7 +765,7 @@
         <v>2008</v>
       </c>
       <c r="D17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -773,7 +779,7 @@
         <v>2009</v>
       </c>
       <c r="D18" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -787,7 +793,7 @@
         <v>2010</v>
       </c>
       <c r="D19" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -801,7 +807,7 @@
         <v>2011</v>
       </c>
       <c r="D20" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -815,7 +821,7 @@
         <v>2012</v>
       </c>
       <c r="D21" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -829,7 +835,7 @@
         <v>2013</v>
       </c>
       <c r="D22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -843,7 +849,7 @@
         <v>2014</v>
       </c>
       <c r="D23" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -857,7 +863,7 @@
         <v>2015</v>
       </c>
       <c r="D24" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -871,7 +877,7 @@
         <v>2016</v>
       </c>
       <c r="D25" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -885,7 +891,7 @@
         <v>2017</v>
       </c>
       <c r="D26" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -899,7 +905,7 @@
         <v>2018</v>
       </c>
       <c r="D27" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -913,7 +919,7 @@
         <v>2019</v>
       </c>
       <c r="D28" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -927,7 +933,7 @@
         <v>2020</v>
       </c>
       <c r="D29" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -941,7 +947,7 @@
         <v>2021</v>
       </c>
       <c r="D30" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -955,7 +961,7 @@
         <v>2003</v>
       </c>
       <c r="D31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -969,7 +975,7 @@
         <v>2008</v>
       </c>
       <c r="D32" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -983,7 +989,7 @@
         <v>2013</v>
       </c>
       <c r="D33" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -997,7 +1003,7 @@
         <v>2018</v>
       </c>
       <c r="D34" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -1008,10 +1014,10 @@
         <v>13</v>
       </c>
       <c r="C35">
-        <v>2016</v>
+        <v>2012</v>
       </c>
       <c r="D35" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -1022,10 +1028,24 @@
         <v>14</v>
       </c>
       <c r="C36">
+        <v>2016</v>
+      </c>
+      <c r="D36" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" t="s">
+        <v>7</v>
+      </c>
+      <c r="B37" t="s">
+        <v>15</v>
+      </c>
+      <c r="C37">
         <v>2017</v>
       </c>
-      <c r="D36" t="s">
-        <v>49</v>
+      <c r="D37" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>